<commit_message>
fix skip issues to fit their rigid assessment
</commit_message>
<xml_diff>
--- a/PEWI Budgets 2024$ - 2025$ (021425).xlsx
+++ b/PEWI Budgets 2024$ - 2025$ (021425).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my_pewi\PEWI-People-in-Ecosystem-and-Watershed-Integration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D18FFD-D5DB-4567-8F97-CBB1B2BA830D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4508143-4D74-46FC-B54E-A32215842C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{2A59C1DF-064D-264D-B5F5-440AD859B569}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" activeTab="2" xr2:uid="{2A59C1DF-064D-264D-B5F5-440AD859B569}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions &amp; summary data" sheetId="19" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1775" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1785" uniqueCount="583">
   <si>
     <t>Ag Decision Maker -- Iowa State University Extension and Outreach</t>
   </si>
@@ -2140,31 +2140,13 @@
     <t>500 Acres</t>
   </si>
   <si>
-    <t>Land use</t>
-  </si>
-  <si>
-    <t>Unit price</t>
-  </si>
-  <si>
     <t>Source</t>
   </si>
   <si>
-    <t>Conventional Soybean</t>
-  </si>
-  <si>
     <t>Switchgrass Bioenergy</t>
   </si>
   <si>
     <t>Short-Rotation Woody Biomass</t>
-  </si>
-  <si>
-    <t>Soybean following Corn</t>
-  </si>
-  <si>
-    <t>Corn following Soybean</t>
-  </si>
-  <si>
-    <t>Corn following Corn</t>
   </si>
   <si>
     <t>Carbon Credit</t>
@@ -2203,7 +2185,43 @@
     </r>
   </si>
   <si>
-    <t>Kg −1</t>
+    <r>
+      <t xml:space="preserve">Acre </t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>−1</t>
+    </r>
+  </si>
+  <si>
+    <t>(Johanns, 2024)</t>
+  </si>
+  <si>
+    <t>Land Use Category</t>
+  </si>
+  <si>
+    <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Conventional Corn following Corn</t>
+  </si>
+  <si>
+    <t>Convenetional Corn following Soybean</t>
+  </si>
+  <si>
+    <t>Conventional Soybean following Corn</t>
+  </si>
+  <si>
+    <t>Conventional Conservation Corn</t>
+  </si>
+  <si>
+    <t>USDA, 2025</t>
   </si>
 </sst>
 </file>
@@ -5323,7 +5341,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1E20D6-F156-C447-BE27-5EDB562A8E09}">
-  <dimension ref="B2:M51"/>
+  <dimension ref="B2:M49"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="10.625" customWidth="1"/>
@@ -5820,194 +5838,220 @@
         <v>512</v>
       </c>
     </row>
-    <row r="32" spans="2:9">
+    <row r="32" spans="2:9" ht="16.5" thickBot="1">
       <c r="B32" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="C32" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="D32" t="s">
         <v>183</v>
       </c>
       <c r="E32" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" ht="16.5" thickBot="1">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" ht="16.5" thickBot="1">
       <c r="B33" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" ht="16.5" thickBot="1">
+        <v>578</v>
+      </c>
+      <c r="C33">
+        <v>171.23</v>
+      </c>
+      <c r="D33" s="520" t="s">
+        <v>572</v>
+      </c>
+      <c r="E33" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" ht="16.5" thickBot="1">
       <c r="B34" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="C34">
         <v>171.23</v>
       </c>
       <c r="D34" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4">
+        <v>572</v>
+      </c>
+      <c r="E34" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" ht="16.5" thickBot="1">
       <c r="B35" t="s">
+        <v>580</v>
+      </c>
+      <c r="C35">
+        <v>381.07</v>
+      </c>
+      <c r="D35" s="520" t="s">
+        <v>572</v>
+      </c>
+      <c r="E35" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B36" t="s">
+        <v>581</v>
+      </c>
+      <c r="C36">
+        <v>171.23</v>
+      </c>
+      <c r="D36" s="520" t="s">
+        <v>572</v>
+      </c>
+      <c r="E36" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B37" t="s">
+        <v>458</v>
+      </c>
+      <c r="C37">
+        <v>481.29</v>
+      </c>
+      <c r="D37" s="520" t="s">
+        <v>572</v>
+      </c>
+      <c r="E37" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B38" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38">
+        <v>253</v>
+      </c>
+      <c r="D38" s="520" t="s">
+        <v>572</v>
+      </c>
+      <c r="E38" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B39" t="s">
+        <v>473</v>
+      </c>
+      <c r="C39">
+        <v>180</v>
+      </c>
+      <c r="D39" s="520" t="s">
+        <v>572</v>
+      </c>
+      <c r="E39" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B40" t="s">
+        <v>568</v>
+      </c>
+      <c r="C40">
+        <v>60</v>
+      </c>
+      <c r="D40" s="520" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B41" t="s">
+        <v>569</v>
+      </c>
+      <c r="C41">
+        <v>60</v>
+      </c>
+      <c r="D41" s="520" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B42" t="s">
+        <v>463</v>
+      </c>
+      <c r="C42">
+        <v>12.46</v>
+      </c>
+      <c r="D42" s="520" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5">
+      <c r="B43" t="s">
+        <v>464</v>
+      </c>
+      <c r="C43">
+        <v>12.46</v>
+      </c>
+      <c r="D43" s="520" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5">
+      <c r="B44" t="s">
+        <v>469</v>
+      </c>
+      <c r="C44">
+        <v>0.79</v>
+      </c>
+      <c r="D44" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B45" t="s">
+        <v>470</v>
+      </c>
+      <c r="C45">
+        <v>0.79</v>
+      </c>
+      <c r="D45" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B46" t="s">
+        <v>570</v>
+      </c>
+      <c r="C46">
+        <v>40.82</v>
+      </c>
+      <c r="D46" s="520" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" ht="16.5" thickBot="1">
+      <c r="B47" t="s">
+        <v>467</v>
+      </c>
+      <c r="C47">
+        <v>205</v>
+      </c>
+      <c r="D47" s="520" t="s">
         <v>574</v>
       </c>
-      <c r="C35">
-        <v>171.23</v>
-      </c>
-      <c r="D35" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B36" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B37" t="s">
-        <v>573</v>
-      </c>
-      <c r="C37">
-        <v>381.07</v>
-      </c>
-      <c r="D37" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B38" t="s">
-        <v>456</v>
-      </c>
-      <c r="C38">
-        <v>171.23</v>
-      </c>
-      <c r="D38" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="39" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B39" t="s">
-        <v>458</v>
-      </c>
-      <c r="C39">
-        <v>481.29</v>
-      </c>
-      <c r="D39" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="40" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B40" t="s">
-        <v>131</v>
-      </c>
-      <c r="C40">
-        <v>253</v>
-      </c>
-      <c r="D40" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="41" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B41" t="s">
-        <v>473</v>
-      </c>
-      <c r="C41">
-        <v>180</v>
-      </c>
-      <c r="D41" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="42" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B42" t="s">
+    </row>
+    <row r="48" spans="2:5">
+      <c r="B48" t="s">
+        <v>468</v>
+      </c>
+      <c r="C48">
+        <v>312.08999999999997</v>
+      </c>
+      <c r="D48" s="520" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2">
+      <c r="B49" t="s">
         <v>571</v>
-      </c>
-      <c r="C42">
-        <v>60</v>
-      </c>
-      <c r="D42" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="43" spans="2:4" ht="16.5" thickBot="1">
-      <c r="B43" t="s">
-        <v>572</v>
-      </c>
-      <c r="C43">
-        <v>60</v>
-      </c>
-      <c r="D43" s="520" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="44" spans="2:4">
-      <c r="B44" t="s">
-        <v>463</v>
-      </c>
-      <c r="C44">
-        <v>12.46</v>
-      </c>
-      <c r="D44" s="520" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="45" spans="2:4">
-      <c r="B45" t="s">
-        <v>464</v>
-      </c>
-      <c r="C45">
-        <v>12.46</v>
-      </c>
-      <c r="D45" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="46" spans="2:4">
-      <c r="B46" t="s">
-        <v>469</v>
-      </c>
-      <c r="C46">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="47" spans="2:4">
-      <c r="B47" t="s">
-        <v>470</v>
-      </c>
-      <c r="C47">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="48" spans="2:4">
-      <c r="B48" t="s">
-        <v>576</v>
-      </c>
-      <c r="C48">
-        <v>40.82</v>
-      </c>
-    </row>
-    <row r="49" spans="2:3">
-      <c r="B49" t="s">
-        <v>467</v>
-      </c>
-      <c r="C49">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="50" spans="2:3">
-      <c r="B50" t="s">
-        <v>468</v>
-      </c>
-      <c r="C50">
-        <v>312.08999999999997</v>
-      </c>
-    </row>
-    <row r="51" spans="2:3">
-      <c r="B51" t="s">
-        <v>577</v>
       </c>
     </row>
   </sheetData>
@@ -17091,7 +17135,7 @@
     <row r="77" spans="1:10">
       <c r="A77" s="86">
         <f ca="1">TODAY()</f>
-        <v>45857</v>
+        <v>45859</v>
       </c>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -19814,7 +19858,7 @@
     <row r="101" spans="1:11">
       <c r="A101" s="86">
         <f ca="1">TODAY()</f>
-        <v>45857</v>
+        <v>45859</v>
       </c>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -21424,7 +21468,7 @@
     <row r="73" spans="1:11">
       <c r="A73" s="86">
         <f ca="1">TODAY()</f>
-        <v>45857</v>
+        <v>45859</v>
       </c>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -23198,7 +23242,7 @@
     <row r="88" spans="1:11">
       <c r="A88" s="86">
         <f ca="1">TODAY()</f>
-        <v>45857</v>
+        <v>45859</v>
       </c>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -26175,7 +26219,7 @@
     <row r="133" spans="1:11">
       <c r="A133" s="86">
         <f ca="1">TODAY()</f>
-        <v>45857</v>
+        <v>45859</v>
       </c>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -29133,7 +29177,7 @@
     <row r="133" spans="1:11">
       <c r="A133" s="86">
         <f ca="1">TODAY()</f>
-        <v>45857</v>
+        <v>45859</v>
       </c>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>

</xml_diff>